<commit_message>
updated checkout page of invalid form
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -8,25 +8,26 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PYTHON_DEMOWEBSHOP\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50CDD37C-A2C2-4F29-B4F7-B5DD45A95BCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3A893C7-B021-445D-8C3C-39EECAA6E08C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
     <sheet name="billingForm" sheetId="7" r:id="rId2"/>
-    <sheet name="Recovery" sheetId="2" r:id="rId3"/>
-    <sheet name="CartProducts" sheetId="3" r:id="rId4"/>
-    <sheet name="ValidSearchProducts" sheetId="4" r:id="rId5"/>
-    <sheet name="InvalidSearchProducts" sheetId="5" r:id="rId6"/>
-    <sheet name="Register" sheetId="6" r:id="rId7"/>
+    <sheet name="Invalid billingForm" sheetId="8" r:id="rId3"/>
+    <sheet name="Recovery" sheetId="2" r:id="rId4"/>
+    <sheet name="CartProducts" sheetId="3" r:id="rId5"/>
+    <sheet name="ValidSearchProducts" sheetId="4" r:id="rId6"/>
+    <sheet name="InvalidSearchProducts" sheetId="5" r:id="rId7"/>
+    <sheet name="Register" sheetId="6" r:id="rId8"/>
   </sheets>
   <calcPr calcId="0" iterate="1" iterateCount="1000" iterateDelta="0.01"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="51">
   <si>
     <t>email</t>
   </si>
@@ -819,6 +820,80 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F70F0809-76B0-44A2-BA19-44F6779BA763}">
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="H2">
+        <v>636007</v>
+      </c>
+      <c r="I2">
+        <v>9856739856</v>
+      </c>
+      <c r="J2">
+        <v>555666</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B32614A-1CAD-4D74-8BB3-2A070B01A845}">
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -866,7 +941,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{615DF9EB-CF36-481E-986E-4A842872879F}">
   <dimension ref="A1:A4"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -901,7 +976,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83B2073E-3A15-4BC2-991F-923A6A253721}">
   <dimension ref="A1:A3"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -931,7 +1006,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F23A0BC-81EE-461D-A649-2F0590546996}">
   <dimension ref="A1:A3"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -961,7 +1036,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93C7E778-6F47-4A05-909D-F4B76B0B3A9D}">
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Added Invalid Email Test
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -1,32 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PYTHON_DEMOWEBSHOP\TestData\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50CDD37C-A2C2-4F29-B4F7-B5DD45A95BCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView firstSheet="7" activeTab="7"/>
   </bookViews>
   <sheets>
-    <sheet name="Login" sheetId="1" r:id="rId1"/>
-    <sheet name="billingForm" sheetId="7" r:id="rId2"/>
-    <sheet name="Recovery" sheetId="2" r:id="rId3"/>
-    <sheet name="CartProducts" sheetId="3" r:id="rId4"/>
-    <sheet name="ValidSearchProducts" sheetId="4" r:id="rId5"/>
-    <sheet name="InvalidSearchProducts" sheetId="5" r:id="rId6"/>
-    <sheet name="Register" sheetId="6" r:id="rId7"/>
+    <sheet r:id="rId1" name="Login" sheetId="1"/>
+    <sheet r:id="rId2" name="billingForm" sheetId="2"/>
+    <sheet r:id="rId3" name="Recovery" sheetId="3"/>
+    <sheet r:id="rId4" name="CartProducts" sheetId="4"/>
+    <sheet r:id="rId5" name="ValidSearchProducts" sheetId="5"/>
+    <sheet r:id="rId6" name="InvalidSearchProducts" sheetId="6"/>
+    <sheet r:id="rId7" name="Register" sheetId="7"/>
+    <sheet r:id="rId8" name="InvalidEmail" sheetId="8"/>
   </sheets>
   <calcPr calcId="0" iterate="1" iterateCount="1000" iterateDelta="0.01"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
   <si>
     <t>email</t>
   </si>
@@ -58,6 +52,63 @@
     <t>Login was unsuccessful. Please correct the errors and try again.</t>
   </si>
   <si>
+    <t>Firstname</t>
+  </si>
+  <si>
+    <t>Lastname</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Company</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>City</t>
+  </si>
+  <si>
+    <t>Address1</t>
+  </si>
+  <si>
+    <t>Address2</t>
+  </si>
+  <si>
+    <t>postalcode</t>
+  </si>
+  <si>
+    <t>Phonenumber</t>
+  </si>
+  <si>
+    <t>Faxnumber</t>
+  </si>
+  <si>
+    <t>Jeeva</t>
+  </si>
+  <si>
+    <t>Pranesh</t>
+  </si>
+  <si>
+    <t>Jeeva@gmail.com</t>
+  </si>
+  <si>
+    <t>SmartCliff</t>
+  </si>
+  <si>
+    <t>India</t>
+  </si>
+  <si>
+    <t>Coimbatore</t>
+  </si>
+  <si>
+    <t>RS puram</t>
+  </si>
+  <si>
+    <t>Rs Puram</t>
+  </si>
+  <si>
     <t>message</t>
   </si>
   <si>
@@ -106,9 +157,6 @@
     <t>LastName</t>
   </si>
   <si>
-    <t>Email</t>
-  </si>
-  <si>
     <t>Password</t>
   </si>
   <si>
@@ -121,85 +169,55 @@
     <t xml:space="preserve">K </t>
   </si>
   <si>
+    <t>priyamurugan66</t>
+  </si>
+  <si>
     <t>priya123</t>
   </si>
   <si>
-    <t>priyamurugan66</t>
-  </si>
-  <si>
-    <t>Company</t>
-  </si>
-  <si>
-    <t>City</t>
-  </si>
-  <si>
-    <t>Address1</t>
-  </si>
-  <si>
-    <t>Address2</t>
-  </si>
-  <si>
-    <t>Jeeva</t>
-  </si>
-  <si>
-    <t>Pranesh</t>
-  </si>
-  <si>
-    <t>Jeeva@gmail.com</t>
-  </si>
-  <si>
-    <t>SmartCliff</t>
-  </si>
-  <si>
-    <t>Coimbatore</t>
-  </si>
-  <si>
-    <t>RS puram</t>
-  </si>
-  <si>
-    <t>Rs Puram</t>
-  </si>
-  <si>
-    <t>Firstname</t>
-  </si>
-  <si>
-    <t>Lastname</t>
-  </si>
-  <si>
-    <t>postalcode</t>
-  </si>
-  <si>
-    <t>Phonenumber</t>
-  </si>
-  <si>
-    <t>Faxnumber</t>
-  </si>
-  <si>
-    <t>Country</t>
-  </si>
-  <si>
-    <t>India</t>
+    <t>firstname</t>
+  </si>
+  <si>
+    <t>lastname</t>
+  </si>
+  <si>
+    <t>confirmPassword</t>
+  </si>
+  <si>
+    <t>errorMessage</t>
+  </si>
+  <si>
+    <t>john</t>
+  </si>
+  <si>
+    <t>jack</t>
+  </si>
+  <si>
+    <t>jen</t>
+  </si>
+  <si>
+    <t>jegan</t>
+  </si>
+  <si>
+    <t>jen24</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="11">
     <font>
+      <b val="0"/>
+      <i val="0"/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
+      <b val="0"/>
+      <i val="0"/>
       <u/>
       <sz val="11"/>
       <color theme="10"/>
@@ -208,12 +226,53 @@
     </font>
     <font>
       <b/>
+      <i val="0"/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
     </font>
     <font>
+      <b val="0"/>
+      <i val="0"/>
       <sz val="11"/>
+      <color auto="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <i val="0"/>
+      <sz val="9"/>
+      <color auto="1"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b val="0"/>
+      <i val="0"/>
+      <sz val="9"/>
+      <color auto="1"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b val="0"/>
+      <i val="0"/>
+      <u/>
+      <sz val="9"/>
+      <color theme="10"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b val="0"/>
+      <i val="0"/>
+      <sz val="11"/>
+      <color auto="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="0"/>
+      <i val="0"/>
+      <sz val="9"/>
+      <color rgb="FF555555"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -224,23 +283,6 @@
     <font>
       <sz val="9"/>
       <name val="Segoe UI"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="9"/>
-      <color theme="10"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF555555"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -265,55 +307,54 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
+    <cellStyle name="Normal" xfId="2"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -659,11 +700,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3078386E-4487-4E71-A97E-7D0393C1FFE6}">
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{BE470148-49FC-4F2F-9624-8B6548C20BE9}" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1:H10"/>
+  <sheetFormatPr defaultRowHeight="14.4525" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
-    <row r="1" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="14.25" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -674,7 +715,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -685,7 +726,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -696,14 +737,14 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" ht="14.25" customHeight="1">
       <c r="A5" s="1"/>
       <c r="B5" s="1" t="s">
         <v>4</v>
@@ -712,7 +753,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="115.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" ht="115.5" customHeight="1">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
@@ -722,82 +763,84 @@
       </c>
     </row>
   </sheetData>
+  <printOptions/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait"/>
+  <pageSetup paperSize="1" pageOrder="downThenOver" orientation="portrait"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
     <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
   </headerFooter>
+  <extLst/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3319F672-8F0F-4D5F-B74B-4F6B4654B8B1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{1D4878F1-26C6-48A5-BB56-0B7CCBB38D60}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:K2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
-    <col min="9" max="9" width="11" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.00390625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="B1" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="C1" s="10" t="s">
+    <row r="1" ht="15" customHeight="1">
+      <c r="A1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="E1" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="F1" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="G1" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="H1" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="I1" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="J1" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="K1" s="11" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="B2" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="C2" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="D2" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="E2" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="F2" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="G2" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="H2" s="11" t="s">
-        <v>43</v>
+      <c r="G2" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>28</v>
       </c>
       <c r="I2">
         <v>636007</v>
@@ -811,240 +854,341 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" xr:uid="{42E04894-5B88-4735-AAF2-73D1C145B944}"/>
+    <hyperlink ref="C2" r:id="rId1" display="Jeeva@gmail.com"/>
   </hyperlinks>
+  <printOptions/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B32614A-1CAD-4D74-8BB3-2A070B01A845}">
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait"/>
+  <pageSetup paperSize="1" pageOrder="downThenOver" orientation="portrait"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
     <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
   </headerFooter>
+  <extLst/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{615DF9EB-CF36-481E-986E-4A842872879F}">
-  <dimension ref="A1:A4"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{FC768A81-783A-41A4-8622-B254DC3DCD13}" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1:E15"/>
+  <sheetFormatPr defaultRowHeight="14.4525" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
-    <row r="1" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
-        <v>18</v>
+    <row r="1" ht="14.25" customHeight="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" ht="14.25" customHeight="1">
+      <c r="A2" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" ht="14.25" customHeight="1">
+      <c r="A3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" ht="14.25" customHeight="1">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" display="haritha11@gmail.com"/>
+  </hyperlinks>
+  <printOptions/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait"/>
+  <pageSetup paperSize="1" pageOrder="downThenOver" orientation="portrait"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
     <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
   </headerFooter>
+  <extLst/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83B2073E-3A15-4BC2-991F-923A6A253721}">
-  <dimension ref="A1:A3"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{0D6DE1F9-15A3-4A74-AAAB-40D198D1FEC2}" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1:L21"/>
+  <sheetFormatPr defaultRowHeight="14.4525" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
-    <row r="1" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>21</v>
+    <row r="1" ht="14.25" customHeight="1">
+      <c r="A1" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" ht="14.25" customHeight="1">
+      <c r="A2" s="8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" ht="14.25" customHeight="1">
+      <c r="A3" s="8" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" ht="14.25" customHeight="1">
+      <c r="A4" s="8" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
+  <printOptions/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait"/>
+  <pageSetup paperSize="1" pageOrder="downThenOver" orientation="portrait"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
     <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
   </headerFooter>
+  <extLst/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F23A0BC-81EE-461D-A649-2F0590546996}">
-  <dimension ref="A1:A3"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{4609DCB6-E6EF-491B-86A1-E2494B635AF8}" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr defaultRowHeight="14.4525" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
-    <row r="1" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="14.25" customHeight="1">
       <c r="A1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" ht="14.25" customHeight="1">
       <c r="A2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" ht="14.25" customHeight="1">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
+  <printOptions/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait"/>
+  <pageSetup paperSize="1" pageOrder="downThenOver" orientation="portrait"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
     <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
   </headerFooter>
+  <extLst/>
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{CD58E5B0-C8E1-4613-A4B3-38325CD5840C}" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr defaultRowHeight="14.4525" defaultColWidth="9.140625" customHeight="1"/>
+  <sheetData>
+    <row r="1" ht="14.25" customHeight="1">
+      <c r="A1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" ht="14.25" customHeight="1">
+      <c r="A2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" ht="14.25" customHeight="1">
+      <c r="A3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" pageOrder="downThenOver" orientation="portrait"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
+    <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
+  </headerFooter>
+  <extLst/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93C7E778-6F47-4A05-909D-F4B76B0B3A9D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{C412FA7F-E407-4180-816F-70E02F9326E1}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="19.28515625" customWidth="1"/>
-    <col min="2" max="2" width="14.28515625" customWidth="1"/>
-    <col min="3" max="3" width="30" customWidth="1"/>
+    <col min="1" max="1" width="19.28125" customWidth="1"/>
+    <col min="2" max="2" width="14.28125" customWidth="1"/>
+    <col min="3" max="3" width="30.00390625" customWidth="1"/>
     <col min="4" max="4" width="18.7109375" customWidth="1"/>
     <col min="5" max="5" width="17.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="7"/>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-    </row>
-    <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="7"/>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="9"/>
-    </row>
-    <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="7"/>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-    </row>
-    <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="7"/>
-      <c r="B6" s="7"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
+    <row r="1" ht="15" customHeight="1">
+      <c r="A1" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1">
+      <c r="A2" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1">
+      <c r="A3" s="10"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+    </row>
+    <row r="4" ht="15" customHeight="1">
+      <c r="A4" s="10"/>
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="12"/>
+    </row>
+    <row r="5" ht="15" customHeight="1">
+      <c r="A5" s="10"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+    </row>
+    <row r="6" ht="15" customHeight="1">
+      <c r="A6" s="10"/>
+      <c r="B6" s="10"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" display="priyamurugan66@gmail.com" xr:uid="{00000000-0004-0000-0500-000000000000}"/>
+    <hyperlink ref="C2" r:id="rId1" display="priyamurugan66"/>
   </hyperlinks>
+  <printOptions/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait"/>
+  <pageSetup paperSize="1" pageOrder="downThenOver" orientation="portrait"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
     <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
   </headerFooter>
+  <extLst/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{DF1626C5-9293-4B99-9062-3EB3E44B2E06}" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1:T200"/>
+  <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="13.7109375" customWidth="1"/>
+    <col min="2" max="2" width="13.421875" customWidth="1"/>
+    <col min="3" max="3" width="17.00390625" customWidth="1"/>
+    <col min="4" max="4" width="11.421875" customWidth="1"/>
+    <col min="5" max="5" width="16.8515625" customWidth="1"/>
+    <col min="6" max="6" width="17.00390625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15" customHeight="1">
+      <c r="A1" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1" s="13" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1">
+      <c r="A2" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="B2" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="D2" s="14">
+        <v>123456</v>
+      </c>
+      <c r="E2" s="14">
+        <v>123456</v>
+      </c>
+      <c r="F2" s="14" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1">
+      <c r="A3" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="D3" s="14">
+        <v>987456</v>
+      </c>
+      <c r="E3" s="14">
+        <v>987456</v>
+      </c>
+      <c r="F3" s="14" t="s">
+        <v>32</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" orientation="portrait"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
+    <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
+  </headerFooter>
+  <extLst/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
new test with csv
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -8,21 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PYTHON_DEMOWEBSHOP\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3A893C7-B021-445D-8C3C-39EECAA6E08C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55A9A77A-CC3A-4CB0-B146-20E3E359DCF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
     <sheet name="billingForm" sheetId="7" r:id="rId2"/>
-    <sheet name="Invalid billingForm" sheetId="8" r:id="rId3"/>
-    <sheet name="Recovery" sheetId="2" r:id="rId4"/>
+    <sheet name="Recovery" sheetId="2" r:id="rId3"/>
+    <sheet name="Invalid billingForm" sheetId="9" r:id="rId4"/>
     <sheet name="CartProducts" sheetId="3" r:id="rId5"/>
     <sheet name="ValidSearchProducts" sheetId="4" r:id="rId6"/>
     <sheet name="InvalidSearchProducts" sheetId="5" r:id="rId7"/>
     <sheet name="Register" sheetId="6" r:id="rId8"/>
   </sheets>
-  <calcPr calcId="0" iterate="1" iterateCount="1000" iterateDelta="0.01"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -186,11 +186,18 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -268,9 +275,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -278,28 +285,29 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -820,80 +828,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F70F0809-76B0-44A2-BA19-44F6779BA763}">
-  <dimension ref="A1:J2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="B1" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="C1" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="D1" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="E1" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="F1" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="G1" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="H1" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="I1" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="J1" s="11" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="B2" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="C2" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="D2" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="E2" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="F2" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="G2" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="H2">
-        <v>636007</v>
-      </c>
-      <c r="I2">
-        <v>9856739856</v>
-      </c>
-      <c r="J2">
-        <v>555666</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B32614A-1CAD-4D74-8BB3-2A070B01A845}">
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -938,6 +872,80 @@
     <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
     <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
   </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3127260-5C85-4844-BCC1-CC82E7DF39B5}">
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="I1" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="J1" s="13" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="E2" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="F2" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="G2" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="H2">
+        <v>636007</v>
+      </c>
+      <c r="I2">
+        <v>9856739856</v>
+      </c>
+      <c r="J2">
+        <v>555666</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Added test for Password Mismatch
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
   <bookViews>
-    <workbookView firstSheet="7" activeTab="7"/>
+    <workbookView firstSheet="8" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" name="Login" sheetId="1"/>
@@ -14,13 +14,14 @@
     <sheet r:id="rId6" name="InvalidSearchProducts" sheetId="6"/>
     <sheet r:id="rId7" name="Register" sheetId="7"/>
     <sheet r:id="rId8" name="InvalidEmail" sheetId="8"/>
+    <sheet r:id="rId9" name="PasswordMismatch" sheetId="9"/>
   </sheets>
   <calcPr calcId="0" iterate="1" iterateCount="1000" iterateDelta="0.01"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
   <si>
     <t>email</t>
   </si>
@@ -200,13 +201,19 @@
   </si>
   <si>
     <t>jen24</t>
+  </si>
+  <si>
+    <t>john@gmail.com</t>
+  </si>
+  <si>
+    <t>The password and confirmation password do not match.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -223,6 +230,13 @@
       <color theme="10"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="0"/>
+      <i val="0"/>
+      <sz val="9"/>
+      <color rgb="FF555555"/>
+      <name val="Arial"/>
     </font>
     <font>
       <b/>
@@ -269,13 +283,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="0"/>
-      <i val="0"/>
-      <sz val="9"/>
-      <color rgb="FF555555"/>
-      <name val="Arial"/>
-    </font>
-    <font>
       <b/>
       <sz val="9"/>
       <name val="Segoe UI"/>
@@ -283,6 +290,10 @@
     <font>
       <sz val="9"/>
       <name val="Segoe UI"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -309,10 +320,10 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top"/>
@@ -321,25 +332,25 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0">
@@ -348,10 +359,13 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Normal" xfId="2"/>
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="1"/>
+    <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -700,7 +714,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{BE470148-49FC-4F2F-9624-8B6548C20BE9}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{C61A05BF-4307-470B-A9DC-4CF1A434F686}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="14.4525" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
@@ -775,7 +789,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{1D4878F1-26C6-48A5-BB56-0B7CCBB38D60}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{DACE2658-63FC-42A5-943A-C595E8942F41}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
@@ -868,7 +882,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{FC768A81-783A-41A4-8622-B254DC3DCD13}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{0FE73C91-5630-4FC7-8628-5341DA6DD094}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:E15"/>
   <sheetFormatPr defaultRowHeight="14.4525" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
@@ -918,7 +932,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{0D6DE1F9-15A3-4A74-AAAB-40D198D1FEC2}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{B30BAFA1-30AE-4A2A-A51B-F92394F8E884}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:L21"/>
   <sheetFormatPr defaultRowHeight="14.4525" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
@@ -955,7 +969,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{4609DCB6-E6EF-491B-86A1-E2494B635AF8}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{4DE3A41B-AD8C-43BE-8D3A-EE972D64BA3B}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="14.4525" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
@@ -987,7 +1001,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{CD58E5B0-C8E1-4613-A4B3-38325CD5840C}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{8DB9F02C-DDB0-4EF5-B60A-68FB5BD2639B}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="14.4525" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
@@ -1019,7 +1033,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{C412FA7F-E407-4180-816F-70E02F9326E1}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{76110222-3AFB-4AD5-B391-A722AF9DE27D}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1109,7 +1123,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{DF1626C5-9293-4B99-9062-3EB3E44B2E06}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{40490FA2-07C2-4BA3-BB5B-DAD18F68E4C6}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1122,6 +1136,91 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
+      <c r="A1" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1">
+      <c r="A2" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="D2" s="10">
+        <v>123456</v>
+      </c>
+      <c r="E2" s="10">
+        <v>123456</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1">
+      <c r="A3" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="D3" s="10">
+        <v>987456</v>
+      </c>
+      <c r="E3" s="10">
+        <v>987456</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" pageOrder="downThenOver" orientation="portrait"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
+    <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
+  </headerFooter>
+  <extLst/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{E37C2A13-33F3-43C2-80F6-1FBBAF712010}" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1:T200"/>
+  <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="11.7109375" customWidth="1"/>
+    <col min="2" max="2" width="14.421875" customWidth="1"/>
+    <col min="3" max="3" width="19.28125" customWidth="1"/>
+    <col min="4" max="4" width="11.00390625" customWidth="1"/>
+    <col min="5" max="5" width="17.00390625" customWidth="1"/>
+    <col min="6" max="6" width="15.8515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15" customHeight="1">
       <c r="A1" s="13" t="s">
         <v>51</v>
       </c>
@@ -1141,7 +1240,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1">
+    <row r="2" ht="30.75" customHeight="1">
       <c r="A2" s="14" t="s">
         <v>55</v>
       </c>
@@ -1149,37 +1248,20 @@
         <v>56</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="D2" s="14">
         <v>123456</v>
       </c>
       <c r="E2" s="14">
-        <v>123456</v>
+        <v>654321</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1">
-      <c r="A3" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="B3" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="C3" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="D3" s="14">
-        <v>987456</v>
-      </c>
-      <c r="E3" s="14">
-        <v>987456</v>
-      </c>
-      <c r="F3" s="14" t="s">
-        <v>32</v>
-      </c>
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1">
+      <c r="E4" s="15"/>
     </row>
   </sheetData>
   <printOptions/>

</xml_diff>

<commit_message>
Added existing email test in register module
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
   <bookViews>
-    <workbookView firstSheet="6" activeTab="7"/>
+    <workbookView firstSheet="9" activeTab="9"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" name="Login" sheetId="1"/>
@@ -15,13 +15,14 @@
     <sheet r:id="rId7" name="Register" sheetId="7"/>
     <sheet r:id="rId8" name="InvalidEmail" sheetId="8"/>
     <sheet r:id="rId9" name="PasswordMismatch" sheetId="9"/>
+    <sheet r:id="rId10" name="ExistingEmail" sheetId="10"/>
   </sheets>
   <calcPr calcId="0" iterate="1" iterateCount="1000" iterateDelta="0.01"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="64">
   <si>
     <t>email</t>
   </si>
@@ -207,6 +208,12 @@
   </si>
   <si>
     <t>The password and confirmation password do not match.</t>
+  </si>
+  <si>
+    <t>smith</t>
+  </si>
+  <si>
+    <t>The specified email already exists</t>
   </si>
 </sst>
 </file>
@@ -723,7 +730,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{778EA30C-BACB-42EA-A57E-39DCBD1274F8}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{3F2009E9-7A58-4648-8A88-56D979317780}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="14.4525" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
@@ -797,8 +804,75 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{C8FCE7AA-5FCF-45CF-A1FE-444F5D612252}" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1:T200"/>
+  <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="15.28125" customWidth="1"/>
+    <col min="2" max="2" width="13.57421875" customWidth="1"/>
+    <col min="3" max="3" width="19.421875" customWidth="1"/>
+    <col min="5" max="5" width="17.140625" customWidth="1"/>
+    <col min="6" max="6" width="27.57421875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15" customHeight="1">
+      <c r="A1" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1" s="13" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1">
+      <c r="A2" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="14">
+        <v>123456</v>
+      </c>
+      <c r="E2" s="14">
+        <v>123456</v>
+      </c>
+      <c r="F2" s="14" t="s">
+        <v>63</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" display="haritha11@gmail.com"/>
+  </hyperlinks>
+  <printOptions/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" orientation="portrait"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
+    <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
+  </headerFooter>
+  <extLst/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{FACD525B-E2CC-42C3-8C34-11504C2C1A1C}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{5D09D527-8FE8-4371-BD5C-77B385786984}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
@@ -891,7 +965,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{26D412E1-4B59-44D8-9A2F-1426E2BB32AB}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{902F114B-D21B-4197-8C26-5C3F28C4C1C8}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:E15"/>
   <sheetFormatPr defaultRowHeight="14.4525" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
@@ -941,7 +1015,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{A6CD0CE1-A2C3-4BFB-AA16-EA2007FA0F0A}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{0ADB307D-7DCF-4534-A424-91349B0B0AA2}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:L21"/>
   <sheetFormatPr defaultRowHeight="14.4525" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
@@ -978,7 +1052,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{A286E857-6321-4CE0-B5B6-AE501ED49EF6}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{E2637D49-2103-4005-94AA-28491841A7BC}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="14.4525" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
@@ -1010,7 +1084,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{35C6B6A3-DDDE-4D88-BBB5-152C81BED341}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{4B0755E1-9DE7-4CAE-9AC7-CDD13B30A641}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="14.4525" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
@@ -1042,7 +1116,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{931A8277-7016-4384-AC95-3572276E02C9}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{B4DA45CC-5D9E-42AC-9381-FF892A176435}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1132,7 +1206,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{80278B5F-0306-4648-94C8-8ADD2D81EBDA}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{7E51C887-C433-47E9-A3AA-1E348942DEDB}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1217,7 +1291,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{1699A065-AD9F-4547-83B7-5DC67E2C2EFF}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{8ABA0BD8-C877-42CA-B917-A393B701259B}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>

</xml_diff>

<commit_message>
Added test for giftcard
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
   <bookViews>
-    <workbookView firstSheet="9" activeTab="9"/>
+    <workbookView firstSheet="10" activeTab="11"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" name="Login" sheetId="1"/>
@@ -16,13 +16,16 @@
     <sheet r:id="rId8" name="InvalidEmail" sheetId="8"/>
     <sheet r:id="rId9" name="PasswordMismatch" sheetId="9"/>
     <sheet r:id="rId10" name="ExistingEmail" sheetId="10"/>
+    <sheet r:id="rId11" name="GiftCard" sheetId="11"/>
+    <sheet r:id="rId12" name="InvalidRecipientEmail" sheetId="12"/>
+    <sheet r:id="rId13" name="QuantityUpdate" sheetId="13"/>
   </sheets>
   <calcPr calcId="0" iterate="1" iterateCount="1000" iterateDelta="0.01"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="79">
   <si>
     <t>email</t>
   </si>
@@ -214,13 +217,58 @@
   </si>
   <si>
     <t>The specified email already exists</t>
+  </si>
+  <si>
+    <t>RecipientName</t>
+  </si>
+  <si>
+    <t>RecipientEmail</t>
+  </si>
+  <si>
+    <t>SenderName</t>
+  </si>
+  <si>
+    <t>John</t>
+  </si>
+  <si>
+    <t>jenny04@gmail.com</t>
+  </si>
+  <si>
+    <t>David</t>
+  </si>
+  <si>
+    <t>recipientName</t>
+  </si>
+  <si>
+    <t>recipientEmail</t>
+  </si>
+  <si>
+    <t>senderName</t>
+  </si>
+  <si>
+    <t>Jack</t>
+  </si>
+  <si>
+    <t>Jenny</t>
+  </si>
+  <si>
+    <t>jenny123</t>
+  </si>
+  <si>
+    <t>Smith</t>
+  </si>
+  <si>
+    <t>quantity</t>
+  </si>
+  <si>
+    <t>john04@gmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -290,6 +338,21 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <color auto="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="0"/>
+      <i val="0"/>
+      <sz val="11"/>
+      <color auto="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="9"/>
       <name val="Segoe UI"/>
@@ -303,10 +366,6 @@
       <sz val="9"/>
       <color theme="10"/>
       <name val="Segoe UI"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -366,17 +425,17 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0">
-      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -730,7 +789,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{3F2009E9-7A58-4648-8A88-56D979317780}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{08651FB6-3569-4185-9000-645C221886A2}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="14.4525" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
@@ -805,7 +864,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{C8FCE7AA-5FCF-45CF-A1FE-444F5D612252}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{C4E02243-6D59-42CE-8446-0F24191AC111}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -817,48 +876,95 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="9" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="14">
+      <c r="D2" s="10">
         <v>123456</v>
       </c>
-      <c r="E2" s="14">
+      <c r="E2" s="10">
         <v>123456</v>
       </c>
-      <c r="F2" s="14" t="s">
+      <c r="F2" s="10" t="s">
         <v>63</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" display="haritha11@gmail.com"/>
+  </hyperlinks>
+  <printOptions/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" pageOrder="downThenOver" orientation="portrait"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
+    <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
+  </headerFooter>
+  <extLst/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{73F66714-ADE4-48AF-8436-5920BEA49447}" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1:T200"/>
+  <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="14.7109375" customWidth="1"/>
+    <col min="2" max="2" width="20.00390625" customWidth="1"/>
+    <col min="3" max="3" width="17.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="27.75" customHeight="1">
+      <c r="A1" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1">
+      <c r="A2" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="B2" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>69</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" display="jenny04@gmail.com"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -871,8 +977,141 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{389C38BA-9AB2-4336-815A-249D68288439}" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1:T200"/>
+  <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="12.421875" customWidth="1"/>
+    <col min="2" max="2" width="20.421875" customWidth="1"/>
+    <col min="3" max="3" width="15.140625" customWidth="1"/>
+    <col min="4" max="4" width="21.8515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15" customHeight="1">
+      <c r="A1" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="D1" s="14" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1">
+      <c r="A2" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1">
+      <c r="A3" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>32</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" orientation="portrait"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
+    <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
+  </headerFooter>
+  <extLst/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{D78D3AEB-7632-48CC-9402-8BFC078453ED}" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1:T200"/>
+  <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="19.28125" customWidth="1"/>
+    <col min="2" max="2" width="24.7109375" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15" customHeight="1">
+      <c r="A1" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="D1" s="14" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1">
+      <c r="A2" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="B2" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="D2" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1">
+      <c r="A3" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="B3" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="D3" s="15">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" display="john04@gmail.com"/>
+    <hyperlink ref="B3" r:id="rId2" display="jenny04@gmail.com"/>
+  </hyperlinks>
+  <printOptions/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" orientation="portrait"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
+    <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
+  </headerFooter>
+  <extLst/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{5D09D527-8FE8-4371-BD5C-77B385786984}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{371862CC-2783-4133-9D2B-EC699DD4CB0F}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
@@ -965,7 +1204,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{902F114B-D21B-4197-8C26-5C3F28C4C1C8}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{A905FF21-AAEE-4EF8-A4AE-AA8B414773A9}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:E15"/>
   <sheetFormatPr defaultRowHeight="14.4525" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
@@ -1015,7 +1254,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{0ADB307D-7DCF-4534-A424-91349B0B0AA2}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{1F457C2A-E973-49BF-B353-B7B91A0B33B3}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:L21"/>
   <sheetFormatPr defaultRowHeight="14.4525" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
@@ -1052,7 +1291,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{E2637D49-2103-4005-94AA-28491841A7BC}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{A128D7EA-7DD4-4DCF-87B0-AD14C3D02078}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="14.4525" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
@@ -1084,7 +1323,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{4B0755E1-9DE7-4CAE-9AC7-CDD13B30A641}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{FF96DA66-2B15-47A8-906B-C0D786BCE373}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="14.4525" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
@@ -1116,7 +1355,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{B4DA45CC-5D9E-42AC-9381-FF892A176435}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{BD45CC7A-073F-4C1B-872C-DEBDE0C1D8F4}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1206,7 +1445,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{7E51C887-C433-47E9-A3AA-1E348942DEDB}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{12556E0D-FC79-4667-A14B-F7188E1C567C}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1291,7 +1530,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{8ABA0BD8-C877-42CA-B917-A393B701259B}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{6AD836D8-0200-44D4-ACEB-FA0E9859E37C}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1304,47 +1543,47 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="9" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="2" ht="30.75" customHeight="1">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="D2" s="14">
+      <c r="D2" s="10">
         <v>123456</v>
       </c>
-      <c r="E2" s="14">
+      <c r="E2" s="10">
         <v>654321</v>
       </c>
-      <c r="F2" s="14" t="s">
+      <c r="F2" s="10" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="E4" s="16"/>
+      <c r="E4" s="13"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1352,7 +1591,7 @@
   </hyperlinks>
   <printOptions/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
+  <pageSetup paperSize="1" pageOrder="downThenOver" orientation="portrait"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
     <oddFooter>&amp;L&amp;C&amp;R</oddFooter>

</xml_diff>

<commit_message>
Updated the code for make it working properly
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
   <bookViews>
-    <workbookView firstSheet="12" activeTab="12"/>
+    <workbookView firstSheet="6" activeTab="9"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" name="Login" sheetId="1"/>
@@ -271,7 +271,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="14">
+  <fonts count="10">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -343,32 +343,10 @@
     <font>
       <b val="0"/>
       <i val="0"/>
-      <color auto="1"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="0"/>
-      <i val="0"/>
       <sz val="11"/>
       <color auto="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="9"/>
-      <color theme="10"/>
-      <name val="Segoe UI"/>
     </font>
   </fonts>
   <fills count="3">
@@ -398,7 +376,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top"/>
@@ -428,17 +406,8 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -792,7 +761,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{B19CC92A-465A-4123-BDAD-A316640F21FF}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{BA1A2697-B7F6-493A-A6F8-D0DB39D272A2}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="14.4525" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
@@ -867,7 +836,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{FA412A0C-0ED1-4E9B-B548-3FD9F6056891}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{D0F43D1F-F943-42EA-9A9E-9BCBFBE34818}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -934,7 +903,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{1E3EECEF-39E8-4A4D-9C0B-D4BC0BDA5C18}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{9CC77986-E5CC-4750-B666-4FDB52A6034A}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -944,24 +913,24 @@
   </cols>
   <sheetData>
     <row r="1" ht="27.75" customHeight="1">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="9" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="10" t="s">
         <v>69</v>
       </c>
     </row>
@@ -971,7 +940,7 @@
   </hyperlinks>
   <printOptions/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
+  <pageSetup paperSize="1" pageOrder="downThenOver" orientation="portrait"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
     <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
@@ -981,7 +950,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{8BC15E72-A143-48EF-B70C-E08A9D673605}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{E27C1309-C8BF-43C5-ADE7-5F78FAE1FD1F}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -992,51 +961,51 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="9" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="10" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="10" t="s">
         <v>74</v>
       </c>
     </row>
   </sheetData>
   <printOptions/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
+  <pageSetup paperSize="1" pageOrder="downThenOver" orientation="portrait"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
     <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
@@ -1046,7 +1015,7 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{C05C859E-EFE3-40BC-8141-E4982BE380E1}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{EC641BE5-B905-49E9-BB16-4324DC27B646}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1056,44 +1025,44 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="9" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="D2" s="15">
+      <c r="D2" s="10">
         <v>2</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="D3" s="15">
+      <c r="D3" s="10">
         <v>3</v>
       </c>
     </row>
@@ -1104,7 +1073,7 @@
   </hyperlinks>
   <printOptions/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
+  <pageSetup paperSize="1" pageOrder="downThenOver" orientation="portrait"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
     <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
@@ -1114,7 +1083,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{599570FF-BE82-4A35-A065-553C68E3368D}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{31001B06-85F1-46F8-A01D-491E78BB582F}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
@@ -1207,7 +1176,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{8344216F-EF0B-4D54-A4C6-2F8FD464615F}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{728E4EB8-EED0-4B41-A679-ACBE1DB7AE3E}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:E15"/>
   <sheetFormatPr defaultRowHeight="14.4525" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
@@ -1257,7 +1226,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{9D33DC60-D0EB-40A3-8465-187C41253610}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{94990E72-0F89-463A-92F7-34BB1A925B63}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:L21"/>
   <sheetFormatPr defaultRowHeight="14.4525" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
@@ -1294,7 +1263,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{D9FAFDEC-5428-491F-BECD-D59E9452DD75}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{1099565E-0E25-41C6-A47A-9642033E5165}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="14.4525" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
@@ -1326,7 +1295,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{152E0BBC-A1D7-410B-B2C8-CA0FC448C0A0}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{A5F7E5D8-3E59-4FC8-A053-A27B10809B84}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="14.4525" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
@@ -1358,7 +1327,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{4461AEC5-A94F-4EFA-A2DA-6A3CAA8DBA81}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{C890C9CB-BD66-45A0-858A-528DDB9177B3}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1448,7 +1417,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{83B1D639-3E4F-469D-8029-6967412CE5DE}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{30FEC90A-C340-4757-BFA2-39A8D41E5274}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1533,7 +1502,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{12BC4A6B-9D4C-4C27-9CC4-5265F2A05671}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{78EC5C9E-DDE0-4271-9C75-644C2A4CAB73}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1542,7 +1511,7 @@
     <col min="3" max="3" width="19.28125" customWidth="1"/>
     <col min="4" max="4" width="11.00390625" customWidth="1"/>
     <col min="5" max="5" width="17.00390625" customWidth="1"/>
-    <col min="6" max="6" width="15.8515625" customWidth="1"/>
+    <col min="6" max="6" width="32.8515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">

</xml_diff>

<commit_message>
Updated the failed scenarios
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
   <bookViews>
-    <workbookView firstSheet="6" activeTab="9"/>
+    <workbookView firstSheet="12" activeTab="11"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" name="Login" sheetId="1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="83">
   <si>
     <t>email</t>
   </si>
@@ -228,6 +228,9 @@
     <t>SenderName</t>
   </si>
   <si>
+    <t>SenderEmail</t>
+  </si>
+  <si>
     <t>John</t>
   </si>
   <si>
@@ -237,6 +240,9 @@
     <t>David</t>
   </si>
   <si>
+    <t>david04@gmail.com</t>
+  </si>
+  <si>
     <t>recipientName</t>
   </si>
   <si>
@@ -249,6 +255,9 @@
     <t>Jack</t>
   </si>
   <si>
+    <t>jack@gmail.com</t>
+  </si>
+  <si>
     <t>Enter valid recipient email</t>
   </si>
   <si>
@@ -261,17 +270,17 @@
     <t>Smith</t>
   </si>
   <si>
-    <t>quantity</t>
-  </si>
-  <si>
-    <t>john04@gmail.com</t>
+    <t>smith@gmail.com</t>
+  </si>
+  <si>
+    <t>Quantity</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -348,6 +357,21 @@
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <i val="0"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="0"/>
+      <i val="0"/>
+      <sz val="9"/>
+      <color theme="10"/>
+      <name val="Segoe UI"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -376,7 +400,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top"/>
@@ -408,6 +432,12 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -761,7 +791,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{BA1A2697-B7F6-493A-A6F8-D0DB39D272A2}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{625BF582-D23E-4B39-B14D-2F5C5B487064}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="14.4525" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
@@ -836,7 +866,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{D0F43D1F-F943-42EA-9A9E-9BCBFBE34818}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{E804CBE1-E661-40A0-A3C4-943F44BD3BE8}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -903,13 +933,14 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{9CC77986-E5CC-4750-B666-4FDB52A6034A}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{B2BA9985-6179-4417-A588-C999534B25C2}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
     <col min="2" max="2" width="20.00390625" customWidth="1"/>
     <col min="3" max="3" width="17.140625" customWidth="1"/>
+    <col min="4" max="4" width="22.8515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="27.75" customHeight="1">
@@ -922,21 +953,28 @@
       <c r="C1" s="9" t="s">
         <v>66</v>
       </c>
+      <c r="D1" s="14" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="10" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>69</v>
+        <v>70</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" display="jenny04@gmail.com"/>
+    <hyperlink ref="D2" r:id="rId2" display="david04@gmail.com" tooltip="david04@gmail.com"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -950,7 +988,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{E27C1309-C8BF-43C5-ADE7-5F78FAE1FD1F}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{A15921D6-F134-4BF5-BE0A-0C268269B878}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -958,118 +996,64 @@
     <col min="2" max="2" width="20.421875" customWidth="1"/>
     <col min="3" max="3" width="15.140625" customWidth="1"/>
     <col min="4" max="4" width="21.8515625" customWidth="1"/>
+    <col min="5" max="5" width="26.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="9" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D1" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="E1" s="9" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="10" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B2" s="10" t="s">
         <v>55</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>74</v>
+        <v>75</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="10" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C3" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="E3" s="10" t="s">
         <v>77</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>74</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" pageOrder="downThenOver" orientation="portrait"/>
-  <headerFooter>
-    <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
-    <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
-  </headerFooter>
-  <extLst/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{EC641BE5-B905-49E9-BB16-4324DC27B646}" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:T200"/>
-  <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
-  <cols>
-    <col min="1" max="1" width="19.28125" customWidth="1"/>
-    <col min="2" max="2" width="24.7109375" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="15" customHeight="1">
-      <c r="A1" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="B1" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="C1" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="D1" s="9" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="2" ht="15" customHeight="1">
-      <c r="A2" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="B2" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="D2" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1">
-      <c r="A3" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="B3" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="D3" s="10">
-        <v>3</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" display="john04@gmail.com"/>
-    <hyperlink ref="B3" r:id="rId2" display="jenny04@gmail.com"/>
+    <hyperlink ref="D2" r:id="rId1" display="jack@gmail.com"/>
+    <hyperlink ref="D3" r:id="rId2" display="smith@gmail.com"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1082,8 +1066,76 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{5E116621-ABC2-450C-9C1D-5032D0868FDD}" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1:T200"/>
+  <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="19.28125" customWidth="1"/>
+    <col min="2" max="2" width="24.7109375" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" customWidth="1"/>
+    <col min="4" max="4" width="18.28125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15" customHeight="1">
+      <c r="A1" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1">
+      <c r="A2" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="E2" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1">
+      <c r="A3" s="10"/>
+      <c r="B3" s="11"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="3"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" display="jenny04@gmail.com"/>
+    <hyperlink ref="D2" r:id="rId2" display="david04@gmail.com"/>
+  </hyperlinks>
+  <printOptions/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" pageOrder="downThenOver" orientation="portrait"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
+    <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
+  </headerFooter>
+  <extLst/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{31001B06-85F1-46F8-A01D-491E78BB582F}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{0A4C5796-8ECD-4CE9-8C31-C4F50D44801E}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
@@ -1176,7 +1228,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{728E4EB8-EED0-4B41-A679-ACBE1DB7AE3E}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{FF7572F2-67E3-4FA5-8645-D58F3D3773BA}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:E15"/>
   <sheetFormatPr defaultRowHeight="14.4525" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
@@ -1226,7 +1278,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{94990E72-0F89-463A-92F7-34BB1A925B63}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{08130C6C-FFC4-41E6-A85B-F89DC9F8142A}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:L21"/>
   <sheetFormatPr defaultRowHeight="14.4525" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
@@ -1263,7 +1315,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{1099565E-0E25-41C6-A47A-9642033E5165}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{CB77995D-0275-4A37-9B6B-63016D1A9300}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="14.4525" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
@@ -1295,7 +1347,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{A5F7E5D8-3E59-4FC8-A053-A27B10809B84}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{8925DCB6-7D7F-4381-95D1-83DF1EFF762A}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="14.4525" defaultColWidth="9.140625" customHeight="1"/>
   <sheetData>
@@ -1327,7 +1379,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{C890C9CB-BD66-45A0-858A-528DDB9177B3}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{872D30BC-D205-4A7A-A295-829602537C5A}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1417,7 +1469,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{30FEC90A-C340-4757-BFA2-39A8D41E5274}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{B7EF4247-C249-4F15-8836-D3A83B1605A3}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>
@@ -1502,7 +1554,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{78EC5C9E-DDE0-4271-9C75-644C2A4CAB73}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{BC1D3F98-BE28-43AE-96F3-D303687F9C00}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <cols>

</xml_diff>